<commit_message>
Primer intento para usar missing para actualizar resultados en pagina web
</commit_message>
<xml_diff>
--- a/data/germany/p6_deployment/missing/data_preparation/all/df_integrated_missing.xlsx
+++ b/data/germany/p6_deployment/missing/data_preparation/all/df_integrated_missing.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BN124"/>
+  <dimension ref="A1:BN133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26871,6 +26871,1618 @@
       <c r="BM124" t="inlineStr"/>
       <c r="BN124" t="inlineStr"/>
     </row>
+    <row r="125">
+      <c r="A125" s="1" t="inlineStr">
+        <is>
+          <t>vJqPCEPP</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="n">
+        <v>45508.35416666666</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kampka r 
+  ger </t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">merck stadion am bollenfalltor
+  darmstadt </t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>17810</v>
+      </c>
+      <c r="F125" t="n">
+        <v>17810</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="n">
+        <v>2</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>S0hPB9rA</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>ne1oL3y7</t>
+        </is>
+      </c>
+      <c r="K125" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="L125" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="M125" t="n">
+        <v>47</v>
+      </c>
+      <c r="N125" t="n">
+        <v>53</v>
+      </c>
+      <c r="O125" t="n">
+        <v>11</v>
+      </c>
+      <c r="P125" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>6</v>
+      </c>
+      <c r="R125" t="n">
+        <v>4</v>
+      </c>
+      <c r="S125" t="n">
+        <v>16</v>
+      </c>
+      <c r="T125" t="n">
+        <v>7</v>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>MDhPV0RQ</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>AoL97rX8</t>
+        </is>
+      </c>
+      <c r="W125" t="n">
+        <v>59</v>
+      </c>
+      <c r="X125" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y125" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z125" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>8vndvXTk</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>WG9pOTse</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr"/>
+      <c r="AD125" t="inlineStr"/>
+      <c r="AE125" t="inlineStr"/>
+      <c r="AF125" t="inlineStr"/>
+      <c r="AG125" t="inlineStr"/>
+      <c r="AH125" t="inlineStr"/>
+      <c r="AI125" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="AJ125" t="n">
+        <v>183.3</v>
+      </c>
+      <c r="AK125" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL125" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="AM125" t="n">
+        <v>2490000</v>
+      </c>
+      <c r="AN125" t="n">
+        <v>74</v>
+      </c>
+      <c r="AO125" t="n">
+        <v>25.6875</v>
+      </c>
+      <c r="AP125" t="n">
+        <v>186.25</v>
+      </c>
+      <c r="AQ125" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR125" t="n">
+        <v>68.75</v>
+      </c>
+      <c r="AS125" t="n">
+        <v>1679687.5</v>
+      </c>
+      <c r="AT125" t="n">
+        <v>73.1875</v>
+      </c>
+      <c r="AU125" t="n">
+        <v>21.95454545454545</v>
+      </c>
+      <c r="AV125" t="n">
+        <v>186.4545454545455</v>
+      </c>
+      <c r="AW125" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX125" t="n">
+        <v>64.04545454545455</v>
+      </c>
+      <c r="AY125" t="n">
+        <v>1346590.909090909</v>
+      </c>
+      <c r="AZ125" t="n">
+        <v>72.95454545454545</v>
+      </c>
+      <c r="BA125" t="inlineStr"/>
+      <c r="BB125" t="inlineStr"/>
+      <c r="BC125" t="inlineStr"/>
+      <c r="BD125" t="inlineStr"/>
+      <c r="BE125" t="inlineStr"/>
+      <c r="BF125" t="inlineStr"/>
+      <c r="BG125" t="inlineStr"/>
+      <c r="BH125" t="inlineStr"/>
+      <c r="BI125" t="inlineStr"/>
+      <c r="BJ125" t="inlineStr"/>
+      <c r="BK125" t="inlineStr"/>
+      <c r="BL125" t="inlineStr"/>
+      <c r="BM125" t="inlineStr"/>
+      <c r="BN125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="inlineStr">
+        <is>
+          <t>2Hl43AnC</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="n">
+        <v>45508.35416666666</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hempel r 
+  ger </t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sportpark ronhof thomas sommer
+  furth </t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>16626</v>
+      </c>
+      <c r="F126" t="n">
+        <v>12664</v>
+      </c>
+      <c r="G126" t="n">
+        <v>3</v>
+      </c>
+      <c r="H126" t="n">
+        <v>1</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>CCQGbik8</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>zedZaSL7</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="L126" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="M126" t="n">
+        <v>47</v>
+      </c>
+      <c r="N126" t="n">
+        <v>53</v>
+      </c>
+      <c r="O126" t="n">
+        <v>22</v>
+      </c>
+      <c r="P126" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>9</v>
+      </c>
+      <c r="R126" t="n">
+        <v>5</v>
+      </c>
+      <c r="S126" t="n">
+        <v>9</v>
+      </c>
+      <c r="T126" t="n">
+        <v>11</v>
+      </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>8E86CPuD</t>
+        </is>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>pdPRS0me</t>
+        </is>
+      </c>
+      <c r="W126" t="n">
+        <v>59</v>
+      </c>
+      <c r="X126" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z126" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>6FDqshzF</t>
+        </is>
+      </c>
+      <c r="AB126" t="inlineStr"/>
+      <c r="AC126" t="n">
+        <v>25</v>
+      </c>
+      <c r="AD126" t="n">
+        <v>183.1</v>
+      </c>
+      <c r="AE126" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF126" t="n">
+        <v>67</v>
+      </c>
+      <c r="AG126" t="n">
+        <v>1480000</v>
+      </c>
+      <c r="AH126" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="AI126" t="inlineStr"/>
+      <c r="AJ126" t="inlineStr"/>
+      <c r="AK126" t="inlineStr"/>
+      <c r="AL126" t="inlineStr"/>
+      <c r="AM126" t="inlineStr"/>
+      <c r="AN126" t="inlineStr"/>
+      <c r="AO126" t="n">
+        <v>22.72727272727273</v>
+      </c>
+      <c r="AP126" t="n">
+        <v>182.5454545454545</v>
+      </c>
+      <c r="AQ126" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR126" t="n">
+        <v>64.59090909090909</v>
+      </c>
+      <c r="AS126" t="n">
+        <v>1273863.636363636</v>
+      </c>
+      <c r="AT126" t="n">
+        <v>72.86363636363636</v>
+      </c>
+      <c r="AU126" t="n">
+        <v>25.57142857142857</v>
+      </c>
+      <c r="AV126" t="n">
+        <v>181.8571428571429</v>
+      </c>
+      <c r="AW126" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX126" t="n">
+        <v>66.71428571428571</v>
+      </c>
+      <c r="AY126" t="n">
+        <v>1175000</v>
+      </c>
+      <c r="AZ126" t="n">
+        <v>68.42857142857143</v>
+      </c>
+      <c r="BA126" t="inlineStr"/>
+      <c r="BB126" t="inlineStr"/>
+      <c r="BC126" t="inlineStr"/>
+      <c r="BD126" t="inlineStr"/>
+      <c r="BE126" t="inlineStr"/>
+      <c r="BF126" t="inlineStr"/>
+      <c r="BG126" t="inlineStr"/>
+      <c r="BH126" t="inlineStr"/>
+      <c r="BI126" t="inlineStr"/>
+      <c r="BJ126" t="inlineStr"/>
+      <c r="BK126" t="inlineStr"/>
+      <c r="BL126" t="inlineStr"/>
+      <c r="BM126" t="inlineStr"/>
+      <c r="BN126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="inlineStr">
+        <is>
+          <t>SIOxI915</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="n">
+        <v>45508.35416666666</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">schroder r 
+  ger </t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">donaustadion
+  ulm </t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>19500</v>
+      </c>
+      <c r="F127" t="n">
+        <v>17400</v>
+      </c>
+      <c r="G127" t="n">
+        <v>1</v>
+      </c>
+      <c r="H127" t="n">
+        <v>2</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>tbC3EcQn</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>naWckLmC</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L127" t="n">
+        <v>3</v>
+      </c>
+      <c r="M127" t="n">
+        <v>54</v>
+      </c>
+      <c r="N127" t="n">
+        <v>46</v>
+      </c>
+      <c r="O127" t="n">
+        <v>12</v>
+      </c>
+      <c r="P127" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>3</v>
+      </c>
+      <c r="R127" t="n">
+        <v>4</v>
+      </c>
+      <c r="S127" t="n">
+        <v>12</v>
+      </c>
+      <c r="T127" t="n">
+        <v>16</v>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>QevvB2nf</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>4bJLk19p</t>
+        </is>
+      </c>
+      <c r="W127" t="n">
+        <v>59</v>
+      </c>
+      <c r="X127" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y127" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z127" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA127" t="inlineStr"/>
+      <c r="AB127" t="inlineStr"/>
+      <c r="AC127" t="inlineStr"/>
+      <c r="AD127" t="inlineStr"/>
+      <c r="AE127" t="inlineStr"/>
+      <c r="AF127" t="inlineStr"/>
+      <c r="AG127" t="inlineStr"/>
+      <c r="AH127" t="inlineStr"/>
+      <c r="AI127" t="n">
+        <v>25</v>
+      </c>
+      <c r="AJ127" t="n">
+        <v>184.6363636363636</v>
+      </c>
+      <c r="AK127" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL127" t="n">
+        <v>67.63636363636364</v>
+      </c>
+      <c r="AM127" t="n">
+        <v>1484090.909090909</v>
+      </c>
+      <c r="AN127" t="n">
+        <v>70.63636363636364</v>
+      </c>
+      <c r="AO127" t="inlineStr"/>
+      <c r="AP127" t="inlineStr"/>
+      <c r="AQ127" t="inlineStr"/>
+      <c r="AR127" t="inlineStr"/>
+      <c r="AS127" t="inlineStr"/>
+      <c r="AT127" t="inlineStr"/>
+      <c r="AU127" t="n">
+        <v>25.22222222222222</v>
+      </c>
+      <c r="AV127" t="n">
+        <v>180.9444444444445</v>
+      </c>
+      <c r="AW127" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX127" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="AY127" t="n">
+        <v>1468055.555555556</v>
+      </c>
+      <c r="AZ127" t="n">
+        <v>71.11111111111111</v>
+      </c>
+      <c r="BA127" t="inlineStr"/>
+      <c r="BB127" t="inlineStr"/>
+      <c r="BC127" t="inlineStr"/>
+      <c r="BD127" t="inlineStr"/>
+      <c r="BE127" t="inlineStr"/>
+      <c r="BF127" t="inlineStr"/>
+      <c r="BG127" t="inlineStr"/>
+      <c r="BH127" t="inlineStr"/>
+      <c r="BI127" t="inlineStr"/>
+      <c r="BJ127" t="inlineStr"/>
+      <c r="BK127" t="inlineStr"/>
+      <c r="BL127" t="inlineStr"/>
+      <c r="BM127" t="inlineStr"/>
+      <c r="BN127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="inlineStr">
+        <is>
+          <t>EeIMLi2t</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="n">
+        <v>45507.64583333334</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stieler t 
+  ger </t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">veltins arena
+  gelsenkirchen </t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>62271</v>
+      </c>
+      <c r="F128" t="n">
+        <v>61000</v>
+      </c>
+      <c r="G128" t="n">
+        <v>5</v>
+      </c>
+      <c r="H128" t="n">
+        <v>1</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>0Ija0Ej9</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>QqLCC3il</t>
+        </is>
+      </c>
+      <c r="K128" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="L128" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="M128" t="n">
+        <v>52</v>
+      </c>
+      <c r="N128" t="n">
+        <v>48</v>
+      </c>
+      <c r="O128" t="n">
+        <v>14</v>
+      </c>
+      <c r="P128" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>8</v>
+      </c>
+      <c r="R128" t="n">
+        <v>5</v>
+      </c>
+      <c r="S128" t="n">
+        <v>13</v>
+      </c>
+      <c r="T128" t="n">
+        <v>11</v>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>txZLBQVC</t>
+        </is>
+      </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>SQrxFAMl</t>
+        </is>
+      </c>
+      <c r="W128" t="n">
+        <v>59</v>
+      </c>
+      <c r="X128" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y128" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z128" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>nP1i5US1</t>
+        </is>
+      </c>
+      <c r="AB128" t="inlineStr">
+        <is>
+          <t>dfNCCCzS</t>
+        </is>
+      </c>
+      <c r="AC128" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="AD128" t="n">
+        <v>187.125</v>
+      </c>
+      <c r="AE128" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF128" t="n">
+        <v>69</v>
+      </c>
+      <c r="AG128" t="n">
+        <v>1740625</v>
+      </c>
+      <c r="AH128" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="AI128" t="n">
+        <v>25.375</v>
+      </c>
+      <c r="AJ128" t="n">
+        <v>183.25</v>
+      </c>
+      <c r="AK128" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="AL128" t="n">
+        <v>66.875</v>
+      </c>
+      <c r="AM128" t="n">
+        <v>1287500</v>
+      </c>
+      <c r="AN128" t="n">
+        <v>71.875</v>
+      </c>
+      <c r="AO128" t="n">
+        <v>27.22222222222222</v>
+      </c>
+      <c r="AP128" t="n">
+        <v>190.2222222222222</v>
+      </c>
+      <c r="AQ128" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR128" t="n">
+        <v>67.94444444444444</v>
+      </c>
+      <c r="AS128" t="n">
+        <v>1294444.444444444</v>
+      </c>
+      <c r="AT128" t="n">
+        <v>70.88888888888889</v>
+      </c>
+      <c r="AU128" t="n">
+        <v>24.57142857142857</v>
+      </c>
+      <c r="AV128" t="n">
+        <v>184.9285714285714</v>
+      </c>
+      <c r="AW128" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX128" t="n">
+        <v>66.07142857142857</v>
+      </c>
+      <c r="AY128" t="n">
+        <v>1302142.857142857</v>
+      </c>
+      <c r="AZ128" t="n">
+        <v>71.14285714285714</v>
+      </c>
+      <c r="BA128" t="inlineStr"/>
+      <c r="BB128" t="inlineStr"/>
+      <c r="BC128" t="inlineStr"/>
+      <c r="BD128" t="inlineStr"/>
+      <c r="BE128" t="inlineStr"/>
+      <c r="BF128" t="inlineStr"/>
+      <c r="BG128" t="inlineStr"/>
+      <c r="BH128" t="inlineStr"/>
+      <c r="BI128" t="inlineStr"/>
+      <c r="BJ128" t="inlineStr"/>
+      <c r="BK128" t="inlineStr"/>
+      <c r="BL128" t="inlineStr"/>
+      <c r="BM128" t="inlineStr"/>
+      <c r="BN128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="inlineStr">
+        <is>
+          <t>fiod5WHa</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="n">
+        <v>45507.33333333334</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bacher m 
+  ger </t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heinz von heiden arena
+  hannover </t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>49200</v>
+      </c>
+      <c r="F129" t="n">
+        <v>31800</v>
+      </c>
+      <c r="G129" t="n">
+        <v>2</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>dfNCCCzS</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>UiCmEP56</t>
+        </is>
+      </c>
+      <c r="K129" t="n">
+        <v>2</v>
+      </c>
+      <c r="L129" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="M129" t="n">
+        <v>58</v>
+      </c>
+      <c r="N129" t="n">
+        <v>42</v>
+      </c>
+      <c r="O129" t="n">
+        <v>16</v>
+      </c>
+      <c r="P129" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>5</v>
+      </c>
+      <c r="R129" t="n">
+        <v>3</v>
+      </c>
+      <c r="S129" t="n">
+        <v>12</v>
+      </c>
+      <c r="T129" t="n">
+        <v>17</v>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>t0ZPdkUl</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>zyLSrbZQ</t>
+        </is>
+      </c>
+      <c r="W129" t="n">
+        <v>59</v>
+      </c>
+      <c r="X129" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y129" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z129" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>QqLCC3il</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr"/>
+      <c r="AC129" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="AD129" t="n">
+        <v>184.3</v>
+      </c>
+      <c r="AE129" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AF129" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="AG129" t="n">
+        <v>2082500</v>
+      </c>
+      <c r="AH129" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="AI129" t="inlineStr"/>
+      <c r="AJ129" t="inlineStr"/>
+      <c r="AK129" t="inlineStr"/>
+      <c r="AL129" t="inlineStr"/>
+      <c r="AM129" t="inlineStr"/>
+      <c r="AN129" t="inlineStr"/>
+      <c r="AO129" t="n">
+        <v>24.40909090909091</v>
+      </c>
+      <c r="AP129" t="n">
+        <v>183.4545454545455</v>
+      </c>
+      <c r="AQ129" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR129" t="n">
+        <v>68</v>
+      </c>
+      <c r="AS129" t="n">
+        <v>1812500</v>
+      </c>
+      <c r="AT129" t="n">
+        <v>72.81818181818181</v>
+      </c>
+      <c r="AU129" t="inlineStr"/>
+      <c r="AV129" t="inlineStr"/>
+      <c r="AW129" t="inlineStr"/>
+      <c r="AX129" t="inlineStr"/>
+      <c r="AY129" t="inlineStr"/>
+      <c r="AZ129" t="inlineStr"/>
+      <c r="BA129" t="inlineStr"/>
+      <c r="BB129" t="inlineStr"/>
+      <c r="BC129" t="inlineStr"/>
+      <c r="BD129" t="inlineStr"/>
+      <c r="BE129" t="inlineStr"/>
+      <c r="BF129" t="inlineStr"/>
+      <c r="BG129" t="inlineStr"/>
+      <c r="BH129" t="inlineStr"/>
+      <c r="BI129" t="inlineStr"/>
+      <c r="BJ129" t="inlineStr"/>
+      <c r="BK129" t="inlineStr"/>
+      <c r="BL129" t="inlineStr"/>
+      <c r="BM129" t="inlineStr"/>
+      <c r="BN129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="inlineStr">
+        <is>
+          <t>OWxD1lHO</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="n">
+        <v>45507.33333333334</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">haslberger w 
+  ger </t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">olympiastadion
+  berlin </t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>74667</v>
+      </c>
+      <c r="F130" t="n">
+        <v>48591</v>
+      </c>
+      <c r="G130" t="n">
+        <v>1</v>
+      </c>
+      <c r="H130" t="n">
+        <v>2</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2y0u8Wrq</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>G2Op923t</t>
+        </is>
+      </c>
+      <c r="K130" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L130" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M130" t="n">
+        <v>57</v>
+      </c>
+      <c r="N130" t="n">
+        <v>43</v>
+      </c>
+      <c r="O130" t="n">
+        <v>10</v>
+      </c>
+      <c r="P130" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>3</v>
+      </c>
+      <c r="R130" t="n">
+        <v>5</v>
+      </c>
+      <c r="S130" t="n">
+        <v>16</v>
+      </c>
+      <c r="T130" t="n">
+        <v>7</v>
+      </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>YmfcAeCo</t>
+        </is>
+      </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>0AI1QUJH</t>
+        </is>
+      </c>
+      <c r="W130" t="n">
+        <v>59</v>
+      </c>
+      <c r="X130" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y130" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z130" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA130" t="inlineStr"/>
+      <c r="AB130" t="inlineStr"/>
+      <c r="AC130" t="n">
+        <v>23.22222222222222</v>
+      </c>
+      <c r="AD130" t="n">
+        <v>183.7777777777778</v>
+      </c>
+      <c r="AE130" t="n">
+        <v>1.111111111111111</v>
+      </c>
+      <c r="AF130" t="n">
+        <v>69.44444444444444</v>
+      </c>
+      <c r="AG130" t="n">
+        <v>2422222.222222222</v>
+      </c>
+      <c r="AH130" t="n">
+        <v>76.11111111111111</v>
+      </c>
+      <c r="AI130" t="n">
+        <v>25.125</v>
+      </c>
+      <c r="AJ130" t="n">
+        <v>183.625</v>
+      </c>
+      <c r="AK130" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL130" t="n">
+        <v>67</v>
+      </c>
+      <c r="AM130" t="n">
+        <v>1356250</v>
+      </c>
+      <c r="AN130" t="n">
+        <v>72</v>
+      </c>
+      <c r="AO130" t="n">
+        <v>23.55</v>
+      </c>
+      <c r="AP130" t="n">
+        <v>184.2</v>
+      </c>
+      <c r="AQ130" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AR130" t="n">
+        <v>69.25</v>
+      </c>
+      <c r="AS130" t="n">
+        <v>2360000</v>
+      </c>
+      <c r="AT130" t="n">
+        <v>74.75</v>
+      </c>
+      <c r="AU130" t="n">
+        <v>24.9375</v>
+      </c>
+      <c r="AV130" t="n">
+        <v>186.1875</v>
+      </c>
+      <c r="AW130" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX130" t="n">
+        <v>66.9375</v>
+      </c>
+      <c r="AY130" t="n">
+        <v>1417187.5</v>
+      </c>
+      <c r="AZ130" t="n">
+        <v>72.125</v>
+      </c>
+      <c r="BA130" t="inlineStr"/>
+      <c r="BB130" t="inlineStr"/>
+      <c r="BC130" t="inlineStr"/>
+      <c r="BD130" t="inlineStr"/>
+      <c r="BE130" t="inlineStr"/>
+      <c r="BF130" t="inlineStr"/>
+      <c r="BG130" t="inlineStr"/>
+      <c r="BH130" t="inlineStr"/>
+      <c r="BI130" t="inlineStr"/>
+      <c r="BJ130" t="inlineStr"/>
+      <c r="BK130" t="inlineStr"/>
+      <c r="BL130" t="inlineStr"/>
+      <c r="BM130" t="inlineStr"/>
+      <c r="BN130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="inlineStr">
+        <is>
+          <t>zkVf7hmm</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="n">
+        <v>45507.33333333334</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">braun r 
+  ger </t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bbbank wildpark
+  karlsruhe </t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>34302</v>
+      </c>
+      <c r="F131" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G131" t="n">
+        <v>3</v>
+      </c>
+      <c r="H131" t="n">
+        <v>2</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>EB3q7jbk</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>6FDqshzF</t>
+        </is>
+      </c>
+      <c r="K131" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="L131" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="M131" t="n">
+        <v>51</v>
+      </c>
+      <c r="N131" t="n">
+        <v>49</v>
+      </c>
+      <c r="O131" t="n">
+        <v>15</v>
+      </c>
+      <c r="P131" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>5</v>
+      </c>
+      <c r="R131" t="n">
+        <v>5</v>
+      </c>
+      <c r="S131" t="n">
+        <v>15</v>
+      </c>
+      <c r="T131" t="n">
+        <v>12</v>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>OzPMRhK3</t>
+        </is>
+      </c>
+      <c r="V131" t="inlineStr">
+        <is>
+          <t>tO31cZrF</t>
+        </is>
+      </c>
+      <c r="W131" t="n">
+        <v>59</v>
+      </c>
+      <c r="X131" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y131" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z131" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA131" t="inlineStr">
+        <is>
+          <t>naWckLmC</t>
+        </is>
+      </c>
+      <c r="AB131" t="inlineStr">
+        <is>
+          <t>CCQGbik8</t>
+        </is>
+      </c>
+      <c r="AC131" t="n">
+        <v>26.27272727272727</v>
+      </c>
+      <c r="AD131" t="n">
+        <v>184.3636363636364</v>
+      </c>
+      <c r="AE131" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF131" t="n">
+        <v>67.81818181818181</v>
+      </c>
+      <c r="AG131" t="n">
+        <v>1395454.545454545</v>
+      </c>
+      <c r="AH131" t="n">
+        <v>71.90909090909091</v>
+      </c>
+      <c r="AI131" t="n">
+        <v>22.77777777777778</v>
+      </c>
+      <c r="AJ131" t="n">
+        <v>182</v>
+      </c>
+      <c r="AK131" t="n">
+        <v>1.111111111111111</v>
+      </c>
+      <c r="AL131" t="n">
+        <v>66</v>
+      </c>
+      <c r="AM131" t="n">
+        <v>1697222.222222222</v>
+      </c>
+      <c r="AN131" t="n">
+        <v>72.55555555555556</v>
+      </c>
+      <c r="AO131" t="n">
+        <v>22.78947368421053</v>
+      </c>
+      <c r="AP131" t="n">
+        <v>181.1052631578947</v>
+      </c>
+      <c r="AQ131" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR131" t="n">
+        <v>64.84210526315789</v>
+      </c>
+      <c r="AS131" t="n">
+        <v>1087894.736842105</v>
+      </c>
+      <c r="AT131" t="n">
+        <v>72.84210526315789</v>
+      </c>
+      <c r="AU131" t="n">
+        <v>27.77777777777778</v>
+      </c>
+      <c r="AV131" t="n">
+        <v>181.2222222222222</v>
+      </c>
+      <c r="AW131" t="n">
+        <v>1.111111111111111</v>
+      </c>
+      <c r="AX131" t="n">
+        <v>67.44444444444444</v>
+      </c>
+      <c r="AY131" t="n">
+        <v>1377777.777777778</v>
+      </c>
+      <c r="AZ131" t="n">
+        <v>70.22222222222223</v>
+      </c>
+      <c r="BA131" t="inlineStr"/>
+      <c r="BB131" t="inlineStr"/>
+      <c r="BC131" t="inlineStr"/>
+      <c r="BD131" t="inlineStr"/>
+      <c r="BE131" t="inlineStr"/>
+      <c r="BF131" t="inlineStr"/>
+      <c r="BG131" t="inlineStr"/>
+      <c r="BH131" t="inlineStr"/>
+      <c r="BI131" t="inlineStr"/>
+      <c r="BJ131" t="inlineStr"/>
+      <c r="BK131" t="inlineStr"/>
+      <c r="BL131" t="inlineStr"/>
+      <c r="BM131" t="inlineStr"/>
+      <c r="BN131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="inlineStr">
+        <is>
+          <t>f5QUJVWh</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="n">
+        <v>45507.33333333334</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heft f 
+  ger </t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mdcc arena
+  magdeburg </t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>30098</v>
+      </c>
+      <c r="F132" t="n">
+        <v>21469</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="n">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>YFuz2RLm</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>6in2Eknb</t>
+        </is>
+      </c>
+      <c r="K132" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="L132" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="M132" t="n">
+        <v>63</v>
+      </c>
+      <c r="N132" t="n">
+        <v>37</v>
+      </c>
+      <c r="O132" t="n">
+        <v>21</v>
+      </c>
+      <c r="P132" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>6</v>
+      </c>
+      <c r="R132" t="n">
+        <v>3</v>
+      </c>
+      <c r="S132" t="n">
+        <v>11</v>
+      </c>
+      <c r="T132" t="n">
+        <v>8</v>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>IgZoGKFn</t>
+        </is>
+      </c>
+      <c r="V132" t="inlineStr">
+        <is>
+          <t>8E8qmw3d</t>
+        </is>
+      </c>
+      <c r="W132" t="n">
+        <v>59</v>
+      </c>
+      <c r="X132" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y132" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z132" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA132" t="inlineStr"/>
+      <c r="AB132" t="inlineStr"/>
+      <c r="AC132" t="inlineStr"/>
+      <c r="AD132" t="inlineStr"/>
+      <c r="AE132" t="inlineStr"/>
+      <c r="AF132" t="inlineStr"/>
+      <c r="AG132" t="inlineStr"/>
+      <c r="AH132" t="inlineStr"/>
+      <c r="AI132" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="AJ132" t="n">
+        <v>182.3</v>
+      </c>
+      <c r="AK132" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL132" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="AM132" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="AN132" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="AO132" t="n">
+        <v>24.93333333333333</v>
+      </c>
+      <c r="AP132" t="n">
+        <v>176.3333333333333</v>
+      </c>
+      <c r="AQ132" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR132" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="AS132" t="n">
+        <v>1375000</v>
+      </c>
+      <c r="AT132" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="AU132" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="AV132" t="n">
+        <v>181.4666666666667</v>
+      </c>
+      <c r="AW132" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX132" t="n">
+        <v>64.93333333333334</v>
+      </c>
+      <c r="AY132" t="n">
+        <v>908333.3333333334</v>
+      </c>
+      <c r="AZ132" t="n">
+        <v>68.26666666666667</v>
+      </c>
+      <c r="BA132" t="inlineStr"/>
+      <c r="BB132" t="inlineStr"/>
+      <c r="BC132" t="inlineStr"/>
+      <c r="BD132" t="inlineStr"/>
+      <c r="BE132" t="inlineStr"/>
+      <c r="BF132" t="inlineStr"/>
+      <c r="BG132" t="inlineStr"/>
+      <c r="BH132" t="inlineStr"/>
+      <c r="BI132" t="inlineStr"/>
+      <c r="BJ132" t="inlineStr"/>
+      <c r="BK132" t="inlineStr"/>
+      <c r="BL132" t="inlineStr"/>
+      <c r="BM132" t="inlineStr"/>
+      <c r="BN132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="inlineStr">
+        <is>
+          <t>OA1xkBXI</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="n">
+        <v>45506.64583333334</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">burda m 
+  ger </t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rheinenergiestadion
+  cologne </t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F133" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G133" t="n">
+        <v>1</v>
+      </c>
+      <c r="H133" t="n">
+        <v>2</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>WG9pOTse</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>v9k3aY5F</t>
+        </is>
+      </c>
+      <c r="K133" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="L133" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="M133" t="n">
+        <v>58</v>
+      </c>
+      <c r="N133" t="n">
+        <v>42</v>
+      </c>
+      <c r="O133" t="n">
+        <v>26</v>
+      </c>
+      <c r="P133" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>4</v>
+      </c>
+      <c r="R133" t="n">
+        <v>6</v>
+      </c>
+      <c r="S133" t="n">
+        <v>18</v>
+      </c>
+      <c r="T133" t="n">
+        <v>7</v>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>4fX0k7gg</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>EDRZkDzS</t>
+        </is>
+      </c>
+      <c r="W133" t="n">
+        <v>59</v>
+      </c>
+      <c r="X133" t="n">
+        <v>592</v>
+      </c>
+      <c r="Y133" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z133" t="n">
+        <v>20242025</v>
+      </c>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>88HSzjDr</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr">
+        <is>
+          <t>ILyJuN3g</t>
+        </is>
+      </c>
+      <c r="AC133" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="AD133" t="n">
+        <v>186</v>
+      </c>
+      <c r="AE133" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AF133" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="AG133" t="n">
+        <v>4680000</v>
+      </c>
+      <c r="AH133" t="n">
+        <v>79</v>
+      </c>
+      <c r="AI133" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="AJ133" t="n">
+        <v>183.4</v>
+      </c>
+      <c r="AK133" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL133" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="AM133" t="n">
+        <v>2470000</v>
+      </c>
+      <c r="AN133" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="AO133" t="n">
+        <v>25.78947368421053</v>
+      </c>
+      <c r="AP133" t="n">
+        <v>184.7894736842105</v>
+      </c>
+      <c r="AQ133" t="n">
+        <v>1.210526315789474</v>
+      </c>
+      <c r="AR133" t="n">
+        <v>68.63157894736842</v>
+      </c>
+      <c r="AS133" t="n">
+        <v>2486315.789473684</v>
+      </c>
+      <c r="AT133" t="n">
+        <v>73.05263157894737</v>
+      </c>
+      <c r="AU133" t="n">
+        <v>25.25</v>
+      </c>
+      <c r="AV133" t="n">
+        <v>183.25</v>
+      </c>
+      <c r="AW133" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX133" t="n">
+        <v>69.05</v>
+      </c>
+      <c r="AY133" t="n">
+        <v>2124000</v>
+      </c>
+      <c r="AZ133" t="n">
+        <v>72.75</v>
+      </c>
+      <c r="BA133" t="inlineStr"/>
+      <c r="BB133" t="inlineStr"/>
+      <c r="BC133" t="inlineStr"/>
+      <c r="BD133" t="inlineStr"/>
+      <c r="BE133" t="inlineStr"/>
+      <c r="BF133" t="inlineStr"/>
+      <c r="BG133" t="inlineStr"/>
+      <c r="BH133" t="inlineStr"/>
+      <c r="BI133" t="inlineStr"/>
+      <c r="BJ133" t="inlineStr"/>
+      <c r="BK133" t="inlineStr"/>
+      <c r="BL133" t="inlineStr"/>
+      <c r="BM133" t="inlineStr"/>
+      <c r="BN133" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>